<commit_message>
allow searchProband from external hosts
</commit_message>
<xml_diff>
--- a/permission_definitions.xlsx
+++ b/permission_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\configuration\master-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4DDBF5C-A630-42BD-85B2-0060F651530F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC0BB4B-93AB-4777-BC99-B88A0AB7D53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="31890" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="31425" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="permission_definitions_new" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5747" uniqueCount="1491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5745" uniqueCount="1491">
   <si>
     <t>#SERVICE_METHOD</t>
   </si>
@@ -24583,9 +24583,6 @@
       <c r="A1122" t="s">
         <v>1313</v>
       </c>
-      <c r="B1122" t="s">
-        <v>20</v>
-      </c>
       <c r="C1122" t="s">
         <v>1258</v>
       </c>
@@ -24599,9 +24596,6 @@
     <row r="1123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1123" t="s">
         <v>1313</v>
-      </c>
-      <c r="B1123" t="s">
-        <v>20</v>
       </c>
       <c r="G1123" t="s">
         <v>1261</v>

</xml_diff>